<commit_message>
Add LBOMODEL1 per-tab assumptions list (MD/PDF/CSV/TXT)
Publish What/How/Why/Source assumptions for Coversheet, LBO, DCF, Shares,
52wkHL, and ZI_* tabs; sync DCF/Shares inputs to ZoomInfo LBO case.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/LBO/output/vengeanceaiUSC_LBOMODEL1.xlsx
+++ b/LBO/output/vengeanceaiUSC_LBOMODEL1.xlsx
@@ -4794,7 +4794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:M43"/>
+  <dimension ref="B2:M45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -4857,6 +4857,20 @@
       <c r="B43" t="inlineStr">
         <is>
           <t>S&amp;M AI thesis: SG&amp;A margin compressed ~500bps of revenue by Y3 in forecast (see ZI_* tabs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Assumptions list (all tabs): LBO/output/LBOMODEL1_ASSUMPTIONS_LIST.md|.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/vengeanceaiUSC/Rainmaker/cursor/vengeanceaiusclbomodel1-44dc/LBO/output/LBOMODEL1_ASSUMPTIONS_LIST.pdf</t>
         </is>
       </c>
     </row>
@@ -14068,7 +14082,7 @@
     <row r="2" ht="27" customHeight="1" s="244" thickBot="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Discounted Cash Flow Model for BMC</t>
+          <t>Discounted Cash Flow Model for ZoomInfo (GTM) — LBOMODEL1</t>
         </is>
       </c>
       <c r="C2" s="305" t="n"/>
@@ -14105,7 +14119,7 @@
         </is>
       </c>
       <c r="C6" s="511" t="n">
-        <v>46.25</v>
+        <v>5.3875</v>
       </c>
     </row>
     <row r="7">
@@ -14115,7 +14129,7 @@
         </is>
       </c>
       <c r="C7" s="84" t="n">
-        <v>41400</v>
+        <v>46246</v>
       </c>
     </row>
     <row r="8">
@@ -14125,7 +14139,7 @@
         </is>
       </c>
       <c r="C8" s="512" t="n">
-        <v>143.973</v>
+        <v>292.312</v>
       </c>
     </row>
     <row r="9">
@@ -14135,7 +14149,7 @@
         </is>
       </c>
       <c r="C9" s="513" t="n">
-        <v>0.06990222994664612</v>
+        <v>0.0815</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1" s="244" thickBot="1">
@@ -14160,28 +14174,28 @@
         </is>
       </c>
       <c r="C12" s="270" t="n">
-        <v>2011</v>
+        <v>2023</v>
       </c>
       <c r="D12" s="270" t="n">
-        <v>2012</v>
+        <v>2024</v>
       </c>
       <c r="E12" s="270" t="n">
-        <v>2013</v>
+        <v>2025</v>
       </c>
       <c r="F12" s="157" t="n">
-        <v>2014</v>
+        <v>2026</v>
       </c>
       <c r="G12" s="157" t="n">
-        <v>2015</v>
+        <v>2027</v>
       </c>
       <c r="H12" s="157" t="n">
-        <v>2016</v>
+        <v>2028</v>
       </c>
       <c r="I12" s="157" t="n">
-        <v>2017</v>
+        <v>2029</v>
       </c>
       <c r="J12" s="157" t="n">
-        <v>2018</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="13">
@@ -14191,28 +14205,28 @@
         </is>
       </c>
       <c r="C13" s="39" t="n">
-        <v>40633</v>
+        <v>45291</v>
       </c>
       <c r="D13" s="39" t="n">
-        <v>40999</v>
+        <v>45657</v>
       </c>
       <c r="E13" s="39" t="n">
-        <v>41364</v>
+        <v>46022</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>41729</v>
+        <v>46387</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>42094</v>
+        <v>46752</v>
       </c>
       <c r="H13" s="39" t="n">
-        <v>42460</v>
+        <v>47118</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>42825</v>
+        <v>47483</v>
       </c>
       <c r="J13" s="39" t="n">
-        <v>43190</v>
+        <v>47848</v>
       </c>
     </row>
     <row r="14">
@@ -14230,28 +14244,28 @@
         </is>
       </c>
       <c r="C15" s="162" t="n">
-        <v>843.6000000000003</v>
+        <v>340.1</v>
       </c>
       <c r="D15" s="162" t="n">
-        <v>906.4999999999999</v>
+        <v>183.1</v>
       </c>
       <c r="E15" s="162" t="n">
-        <v>882.7000000000003</v>
+        <v>314.5</v>
       </c>
       <c r="F15" s="162" t="n">
-        <v>947.6792413199889</v>
+        <v>359.6</v>
       </c>
       <c r="G15" s="162" t="n">
-        <v>1000.484484594448</v>
+        <v>398</v>
       </c>
       <c r="H15" s="162" t="n">
-        <v>1078.88768747765</v>
+        <v>439.4</v>
       </c>
       <c r="I15" s="162" t="n">
-        <v>1150.07160606407</v>
+        <v>464.4</v>
       </c>
       <c r="J15" s="162" t="n">
-        <v>1226.874119002437</v>
+        <v>478.4</v>
       </c>
     </row>
     <row r="16">
@@ -14261,28 +14275,28 @@
         </is>
       </c>
       <c r="C16" s="162" t="n">
-        <v>532.8000000000003</v>
+        <v>259.5</v>
       </c>
       <c r="D16" s="162" t="n">
-        <v>543.8999999999999</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="E16" s="162" t="n">
-        <v>465.4000000000003</v>
+        <v>225.7</v>
       </c>
       <c r="F16" s="162" t="n">
-        <v>493.6803141804108</v>
+        <v>267.2</v>
       </c>
       <c r="G16" s="162" t="n">
-        <v>559.8040395999167</v>
+        <v>301</v>
       </c>
       <c r="H16" s="162" t="n">
-        <v>634.7919640514119</v>
+        <v>337.6</v>
       </c>
       <c r="I16" s="162" t="n">
-        <v>709.3122632461741</v>
+        <v>358.5</v>
       </c>
       <c r="J16" s="162" t="n">
-        <v>787.9602383046408</v>
+        <v>369.3</v>
       </c>
     </row>
     <row r="17">
@@ -14292,28 +14306,28 @@
         </is>
       </c>
       <c r="C17" s="514" t="n">
-        <v>0.1413514022209673</v>
+        <v>0.21</v>
       </c>
       <c r="D17" s="514" t="n">
-        <v>0.2433962264150944</v>
+        <v>0.21</v>
       </c>
       <c r="E17" s="514" t="n">
-        <v>0.2264547791540078</v>
+        <v>0.21</v>
       </c>
       <c r="F17" s="514" t="n">
-        <v>0.2264547791540078</v>
+        <v>0.21</v>
       </c>
       <c r="G17" s="514" t="n">
-        <v>0.2264547791540078</v>
+        <v>0.21</v>
       </c>
       <c r="H17" s="514" t="n">
-        <v>0.2264547791540078</v>
+        <v>0.21</v>
       </c>
       <c r="I17" s="514" t="n">
-        <v>0.2264547791540078</v>
+        <v>0.21</v>
       </c>
       <c r="J17" s="514" t="n">
-        <v>0.2264547791540078</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="18">
@@ -14323,28 +14337,28 @@
         </is>
       </c>
       <c r="C18" s="71" t="n">
-        <v>457.4879728966689</v>
+        <v>205</v>
       </c>
       <c r="D18" s="71" t="n">
-        <v>411.51679245283</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="E18" s="71" t="n">
-        <v>360.007945781725</v>
+        <v>178.3</v>
       </c>
       <c r="F18" s="71" t="n">
-        <v>381.8840476600047</v>
+        <v>211.1</v>
       </c>
       <c r="G18" s="71" t="n">
-        <v>433.0337394427961</v>
+        <v>237.8</v>
       </c>
       <c r="H18" s="71" t="n">
-        <v>491.0402900234106</v>
+        <v>266.7</v>
       </c>
       <c r="I18" s="71" t="n">
-        <v>548.6851113215323</v>
+        <v>283.2</v>
       </c>
       <c r="J18" s="71" t="n">
-        <v>609.522876557224</v>
+        <v>291.7</v>
       </c>
     </row>
     <row r="19">
@@ -14659,7 +14673,7 @@
         </is>
       </c>
       <c r="J36" s="140" t="n">
-        <v>1226.874119002437</v>
+        <v>478.4</v>
       </c>
     </row>
     <row r="37">
@@ -14677,7 +14691,7 @@
         </is>
       </c>
       <c r="J37" s="412" t="n">
-        <v>7.3</v>
+        <v>8</v>
       </c>
       <c r="K37" s="411" t="n"/>
     </row>
@@ -14804,7 +14818,7 @@
         </is>
       </c>
       <c r="C45" s="162" t="n">
-        <v>179.9999999999991</v>
+        <v>75</v>
       </c>
       <c r="H45" s="400" t="inlineStr">
         <is>
@@ -14829,7 +14843,7 @@
         </is>
       </c>
       <c r="C46" s="162" t="n">
-        <v>5190.276000000002</v>
+        <v>1572.5</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -14851,7 +14865,7 @@
         </is>
       </c>
       <c r="C47" s="71" t="n">
-        <v>5010.276000000003</v>
+        <v>1497.5</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -14875,7 +14889,7 @@
       <c r="F48" s="383" t="n"/>
       <c r="G48" s="383" t="n"/>
       <c r="H48" s="399" t="n">
-        <v>6741.92625</v>
+        <v>1574.8</v>
       </c>
       <c r="I48" s="57" t="n">
         <v>7372.933086845563</v>
@@ -14897,13 +14911,13 @@
         </is>
       </c>
       <c r="H49" s="512" t="n">
-        <v>145.7713783783784</v>
+        <v>292.312</v>
       </c>
       <c r="I49" s="517" t="n">
-        <v>145.7713783783784</v>
+        <v>292.312</v>
       </c>
       <c r="J49" s="517" t="n">
-        <v>145.7713783783784</v>
+        <v>292.312</v>
       </c>
     </row>
     <row r="50">
@@ -14913,7 +14927,7 @@
         </is>
       </c>
       <c r="C50" s="518" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E50" s="383" t="inlineStr">
         <is>
@@ -14921,7 +14935,7 @@
         </is>
       </c>
       <c r="H50" s="519" t="n">
-        <v>46.25</v>
+        <v>5.3875</v>
       </c>
       <c r="I50" s="519" t="n">
         <v>50.57874302119625</v>
@@ -14937,7 +14951,7 @@
         </is>
       </c>
       <c r="C51" s="418" t="n">
-        <v>0.2264547791540078</v>
+        <v>0.21</v>
       </c>
       <c r="E51" s="100" t="inlineStr">
         <is>
@@ -14963,7 +14977,7 @@
         </is>
       </c>
       <c r="C52" s="140" t="n">
-        <v>5010.276000000003</v>
+        <v>1497.5</v>
       </c>
     </row>
     <row r="53">
@@ -14973,7 +14987,7 @@
         </is>
       </c>
       <c r="C53" s="521" t="n">
-        <v>0.7748616857223557</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="55">
@@ -14983,7 +14997,7 @@
         </is>
       </c>
       <c r="C55" s="414" t="n">
-        <v>0.025</v>
+        <v>0.043</v>
       </c>
     </row>
     <row r="56">
@@ -14993,7 +15007,7 @@
         </is>
       </c>
       <c r="C56" s="135" t="n">
-        <v>1.45</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="57">
@@ -15013,7 +15027,7 @@
         </is>
       </c>
       <c r="C58" s="418" t="n">
-        <v>0.2251383142776443</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="59">
@@ -15023,7 +15037,7 @@
         </is>
       </c>
       <c r="C59" s="418" t="n">
-        <v>0.06990222994664612</v>
+        <v>0.0815</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1" s="244" thickBot="1">
@@ -15691,7 +15705,7 @@
     <row r="2" ht="27" customHeight="1" s="244" thickBot="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Diluted shares for BMC</t>
+          <t>Diluted shares for ZoomInfo (GTM) — LBOMODEL1</t>
         </is>
       </c>
       <c r="C2" s="305" t="n"/>
@@ -15715,7 +15729,7 @@
         </is>
       </c>
       <c r="E5" s="496" t="n">
-        <v>46.25</v>
+        <v>5.3875</v>
       </c>
     </row>
     <row r="6">
@@ -15725,7 +15739,7 @@
         </is>
       </c>
       <c r="E6" s="537" t="n">
-        <v>46.25</v>
+        <v>5.3875</v>
       </c>
     </row>
     <row r="7">
@@ -15735,7 +15749,7 @@
         </is>
       </c>
       <c r="E7" s="505" t="n">
-        <v>143.973</v>
+        <v>292.312</v>
       </c>
     </row>
     <row r="8">
@@ -15745,7 +15759,7 @@
         </is>
       </c>
       <c r="E8" s="504" t="n">
-        <v>10.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -15755,7 +15769,7 @@
         </is>
       </c>
       <c r="E9" s="444" t="n">
-        <v>411.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -15765,7 +15779,7 @@
         </is>
       </c>
       <c r="E10" s="444" t="n">
-        <v>8.901621621621622</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -15775,7 +15789,7 @@
         </is>
       </c>
       <c r="E11" s="444" t="n">
-        <v>1.798378378378377</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -15800,7 +15814,7 @@
       </c>
       <c r="D14" s="417" t="n"/>
       <c r="E14" s="444" t="n">
-        <v>145.7713783783784</v>
+        <v>292.312</v>
       </c>
     </row>
     <row r="15">
@@ -15840,13 +15854,13 @@
         <v>1</v>
       </c>
       <c r="C18" s="298" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D18" s="298" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="299" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -15854,13 +15868,13 @@
         <v>2</v>
       </c>
       <c r="C19" s="298" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D19" s="298" t="n">
         <v>18</v>
       </c>
       <c r="E19" s="299" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -15868,13 +15882,13 @@
         <v>3</v>
       </c>
       <c r="C20" s="298" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D20" s="298" t="n">
         <v>22</v>
       </c>
       <c r="E20" s="299" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -15882,13 +15896,13 @@
         <v>4</v>
       </c>
       <c r="C21" s="298" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D21" s="298" t="n">
         <v>28</v>
       </c>
       <c r="E21" s="299" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -15896,13 +15910,13 @@
         <v>5</v>
       </c>
       <c r="C22" s="298" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D22" s="298" t="n">
         <v>32</v>
       </c>
       <c r="E22" s="299" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -15910,13 +15924,13 @@
         <v>6</v>
       </c>
       <c r="C23" s="298" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D23" s="298" t="n">
         <v>36</v>
       </c>
       <c r="E23" s="299" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -15924,13 +15938,13 @@
         <v>7</v>
       </c>
       <c r="C24" s="298" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="D24" s="298" t="n">
         <v>39</v>
       </c>
       <c r="E24" s="299" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -15938,20 +15952,22 @@
         <v>8</v>
       </c>
       <c r="C25" s="298" t="n">
-        <v>7.4</v>
+        <v>0</v>
       </c>
       <c r="D25" s="298" t="n">
         <v>42</v>
       </c>
       <c r="E25" s="299" t="n">
-        <v>7.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="538" t="n">
         <v>9</v>
       </c>
-      <c r="C26" s="298" t="n"/>
+      <c r="C26" s="298" t="n">
+        <v>0</v>
+      </c>
       <c r="D26" s="298" t="n"/>
       <c r="E26" s="299" t="n">
         <v>0</v>
@@ -15961,7 +15977,9 @@
       <c r="B27" s="538" t="n">
         <v>10</v>
       </c>
-      <c r="C27" s="298" t="n"/>
+      <c r="C27" s="298" t="n">
+        <v>0</v>
+      </c>
       <c r="D27" s="298" t="n"/>
       <c r="E27" s="300" t="n">
         <v>0</v>
@@ -15969,7 +15987,7 @@
     </row>
     <row r="28">
       <c r="E28" s="301" t="n">
-        <v>10.7</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -15996,7 +16014,7 @@
     <row r="2" ht="18" customHeight="1" s="244" thickBot="1">
       <c r="A2" s="101" t="inlineStr">
         <is>
-          <t>52 week high low</t>
+          <t>52 week high low — NOTE: tape still sample/legacy; LBOMODEL1 uses GTM $4.31 spot on LBO!D8</t>
         </is>
       </c>
       <c r="B2" s="93" t="n"/>

</xml_diff>

<commit_message>
Add Strategy_Summary commentary, chart, and PDF export
Annotate each Base vs AI metric with commentary, add clustered bar
chart on Strategy_Summary, and publish LBOMODEL1_STRATEGY_SUMMARY.pdf.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/LBO/output/vengeanceaiUSC_LBOMODEL1.xlsx
+++ b/LBO/output/vengeanceaiUSC_LBOMODEL1.xlsx
@@ -93,64 +93,64 @@
     <numFmt numFmtId="187" formatCode="0\A"/>
     <numFmt numFmtId="188" formatCode="General\ &quot;yrs&quot;"/>
     <numFmt numFmtId="189" formatCode="0.000%"/>
-    <numFmt numFmtId="190" formatCode="#,##0.00_);\(#,##0\)"/>
-    <numFmt numFmtId="191" formatCode="#,##0.0%_);\(#,##0.0%\)"/>
-    <numFmt numFmtId="192" formatCode="0.0\ \x"/>
-    <numFmt numFmtId="193" formatCode="#,##0.00\ ;\(#,##0.00\)"/>
-    <numFmt numFmtId="194" formatCode="&quot;$&quot;#,##0.00\ ;\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="195" formatCode="0.0%_);\(0.0%\)"/>
-    <numFmt numFmtId="196" formatCode="0.000\ \x&quot;rate&quot;"/>
-    <numFmt numFmtId="197" formatCode="#,##0.000_);[Red]\(#,##0.000\)"/>
-    <numFmt numFmtId="198" formatCode="0.00_);\(0.00\);0.00"/>
-    <numFmt numFmtId="199" formatCode="\C&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="200" formatCode="#,##0%_);\(#,##0.0%\)"/>
-    <numFmt numFmtId="201" formatCode="_(* #,##0.00000000_);_(* \(#,##0.00000000\);_(* &quot;-&quot;?_);_(@_)"/>
-    <numFmt numFmtId="202" formatCode="mmm\-d\-yyyy"/>
-    <numFmt numFmtId="203" formatCode="mmm\-yyyy"/>
-    <numFmt numFmtId="204" formatCode="yyyy"/>
-    <numFmt numFmtId="205" formatCode="0.00\x&quot;rate&quot;"/>
-    <numFmt numFmtId="206" formatCode="0.0&quot;  &quot;"/>
-    <numFmt numFmtId="207" formatCode="&quot;$&quot;#,##0.0\ ;[Red]\(&quot;$&quot;#,##0\)"/>
-    <numFmt numFmtId="208" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;?_);_(@_)"/>
-    <numFmt numFmtId="209" formatCode="&quot;$&quot;#,##0.000_);[Red]\(&quot;$&quot;#,##0.000\)"/>
-    <numFmt numFmtId="210" formatCode="&quot;$&quot;#,##0.00&quot;A&quot;;[Red]\(&quot;$&quot;#,##0.00\)&quot;A&quot;"/>
-    <numFmt numFmtId="211" formatCode="#,##0.0\ ;[Red]\(&quot;$&quot;#,##0\)"/>
-    <numFmt numFmtId="212" formatCode="&quot;$&quot;#,##0.00&quot;E&quot;;[Red]\(&quot;$&quot;#,##0.00\)&quot;E&quot;"/>
-    <numFmt numFmtId="213" formatCode="_([$€-2]* #,##0.00_);_([$€-2]* \(#,##0.00\);_([$€-2]* &quot;-&quot;??_)"/>
-    <numFmt numFmtId="214" formatCode="#,##0.00;\(#,##0.00\)"/>
-    <numFmt numFmtId="215" formatCode=".%\,\(0.0%%;\t"/>
-    <numFmt numFmtId="216" formatCode="#,##0.0_);[Red]\(#,##0.0\)"/>
-    <numFmt numFmtId="217" formatCode="0.0%_);[Red]\(0.0%\)"/>
-    <numFmt numFmtId="218" formatCode="0.00_);\(0.00\);0.00_)"/>
-    <numFmt numFmtId="219" formatCode="#,##0\x"/>
-    <numFmt numFmtId="220" formatCode="&quot;TKR&quot;\ 0"/>
-    <numFmt numFmtId="221" formatCode=".%\,\(0.%%;\t"/>
-    <numFmt numFmtId="222" formatCode="&quot;$&quot;#,###.0\ \ "/>
-    <numFmt numFmtId="223" formatCode="#,##0.00\x_);[Red]\(#,##0.00\x\)"/>
-    <numFmt numFmtId="224" formatCode="#,##0.000_);\(#,##0.000\)"/>
-    <numFmt numFmtId="225" formatCode="#,##0.00\x_);[Red]\(#,##0.00\x\);&quot;--  &quot;"/>
-    <numFmt numFmtId="226" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="227" formatCode="0.0\x_);[Red]\(0.0\x\)"/>
-    <numFmt numFmtId="228" formatCode="0.0\ "/>
-    <numFmt numFmtId="229" formatCode="&quot;$&quot;#,##0.0;\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="230" formatCode="#,##0.00%_);\(#,##0.00%\)"/>
-    <numFmt numFmtId="231" formatCode="0.00\%;\-0.00\%;0.00\%"/>
-    <numFmt numFmtId="232" formatCode="0.0%\ ;\(0.0%\)"/>
-    <numFmt numFmtId="233" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="234" formatCode="&quot;$&quot;0.00\ "/>
-    <numFmt numFmtId="235" formatCode="0.0\ \ \ \ \ "/>
-    <numFmt numFmtId="236" formatCode="0.00\x;\-0.00\x;0.00\x"/>
-    <numFmt numFmtId="237" formatCode="&quot;$&quot;#,##0.000_);\(&quot;$&quot;#,##0.000\)"/>
-    <numFmt numFmtId="238" formatCode="#,##0.0_);\(#,##0.0\);_(* &quot;-&quot;_)"/>
-    <numFmt numFmtId="239" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="240" formatCode="0.00%_);[Red]\(0.00%\)"/>
-    <numFmt numFmtId="241" formatCode="#,##0.0\x_);\(#,##0.0\x\)"/>
-    <numFmt numFmtId="242" formatCode="#,##0.00\x_);\(#,##0.00\x\)"/>
-    <numFmt numFmtId="243" formatCode="###0&quot;E&quot;_)"/>
-    <numFmt numFmtId="244" formatCode="#,##0.0"/>
-    <numFmt numFmtId="245" formatCode="0.00x"/>
+    <numFmt numFmtId="190" formatCode="#,##0.0"/>
+    <numFmt numFmtId="191" formatCode="0.00x"/>
+    <numFmt numFmtId="192" formatCode="#,##0.00_);\(#,##0\)"/>
+    <numFmt numFmtId="193" formatCode="#,##0.0%_);\(#,##0.0%\)"/>
+    <numFmt numFmtId="194" formatCode="0.0\ \x"/>
+    <numFmt numFmtId="195" formatCode="#,##0.00\ ;\(#,##0.00\)"/>
+    <numFmt numFmtId="196" formatCode="&quot;$&quot;#,##0.00\ ;\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="197" formatCode="0.0%_);\(0.0%\)"/>
+    <numFmt numFmtId="198" formatCode="0.000\ \x&quot;rate&quot;"/>
+    <numFmt numFmtId="199" formatCode="#,##0.000_);[Red]\(#,##0.000\)"/>
+    <numFmt numFmtId="200" formatCode="0.00_);\(0.00\);0.00"/>
+    <numFmt numFmtId="201" formatCode="\C&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="202" formatCode="#,##0%_);\(#,##0.0%\)"/>
+    <numFmt numFmtId="203" formatCode="_(* #,##0.00000000_);_(* \(#,##0.00000000\);_(* &quot;-&quot;?_);_(@_)"/>
+    <numFmt numFmtId="204" formatCode="mmm\-d\-yyyy"/>
+    <numFmt numFmtId="205" formatCode="mmm\-yyyy"/>
+    <numFmt numFmtId="206" formatCode="yyyy"/>
+    <numFmt numFmtId="207" formatCode="0.00\x&quot;rate&quot;"/>
+    <numFmt numFmtId="208" formatCode="0.0&quot;  &quot;"/>
+    <numFmt numFmtId="209" formatCode="&quot;$&quot;#,##0.0\ ;[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="210" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;?_);_(@_)"/>
+    <numFmt numFmtId="211" formatCode="&quot;$&quot;#,##0.000_);[Red]\(&quot;$&quot;#,##0.000\)"/>
+    <numFmt numFmtId="212" formatCode="&quot;$&quot;#,##0.00&quot;A&quot;;[Red]\(&quot;$&quot;#,##0.00\)&quot;A&quot;"/>
+    <numFmt numFmtId="213" formatCode="#,##0.0\ ;[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="214" formatCode="&quot;$&quot;#,##0.00&quot;E&quot;;[Red]\(&quot;$&quot;#,##0.00\)&quot;E&quot;"/>
+    <numFmt numFmtId="215" formatCode="_([$€-2]* #,##0.00_);_([$€-2]* \(#,##0.00\);_([$€-2]* &quot;-&quot;??_)"/>
+    <numFmt numFmtId="216" formatCode="#,##0.00;\(#,##0.00\)"/>
+    <numFmt numFmtId="217" formatCode=".%\,\(0.0%%;\t"/>
+    <numFmt numFmtId="218" formatCode="#,##0.0_);[Red]\(#,##0.0\)"/>
+    <numFmt numFmtId="219" formatCode="0.0%_);[Red]\(0.0%\)"/>
+    <numFmt numFmtId="220" formatCode="0.00_);\(0.00\);0.00_)"/>
+    <numFmt numFmtId="221" formatCode="#,##0\x"/>
+    <numFmt numFmtId="222" formatCode="&quot;TKR&quot;\ 0"/>
+    <numFmt numFmtId="223" formatCode=".%\,\(0.%%;\t"/>
+    <numFmt numFmtId="224" formatCode="&quot;$&quot;#,###.0\ \ "/>
+    <numFmt numFmtId="225" formatCode="#,##0.00\x_);[Red]\(#,##0.00\x\)"/>
+    <numFmt numFmtId="226" formatCode="#,##0.000_);\(#,##0.000\)"/>
+    <numFmt numFmtId="227" formatCode="#,##0.00\x_);[Red]\(#,##0.00\x\);&quot;--  &quot;"/>
+    <numFmt numFmtId="228" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="229" formatCode="0.0\x_);[Red]\(0.0\x\)"/>
+    <numFmt numFmtId="230" formatCode="0.0\ "/>
+    <numFmt numFmtId="231" formatCode="&quot;$&quot;#,##0.0;\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="232" formatCode="#,##0.00%_);\(#,##0.00%\)"/>
+    <numFmt numFmtId="233" formatCode="0.00\%;\-0.00\%;0.00\%"/>
+    <numFmt numFmtId="234" formatCode="0.0%\ ;\(0.0%\)"/>
+    <numFmt numFmtId="235" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="236" formatCode="&quot;$&quot;0.00\ "/>
+    <numFmt numFmtId="237" formatCode="0.0\ \ \ \ \ "/>
+    <numFmt numFmtId="238" formatCode="0.00\x;\-0.00\x;0.00\x"/>
+    <numFmt numFmtId="239" formatCode="&quot;$&quot;#,##0.000_);\(&quot;$&quot;#,##0.000\)"/>
+    <numFmt numFmtId="240" formatCode="#,##0.0_);\(#,##0.0\);_(* &quot;-&quot;_)"/>
+    <numFmt numFmtId="241" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="242" formatCode="0.00%_);[Red]\(0.00%\)"/>
+    <numFmt numFmtId="243" formatCode="#,##0.0\x_);\(#,##0.0\x\)"/>
+    <numFmt numFmtId="244" formatCode="#,##0.00\x_);\(#,##0.00\x\)"/>
+    <numFmt numFmtId="245" formatCode="###0&quot;E&quot;_)"/>
   </numFmts>
-  <fonts count="105">
+  <fonts count="107">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -836,6 +836,15 @@
       <name val="Calibri"/>
       <color rgb="000000FF"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="38">
     <fill>
@@ -1443,19 +1452,19 @@
   <cellStyleXfs count="187">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="190" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="192" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="191" fontId="10" fillId="2" borderId="0"/>
-    <xf numFmtId="192" fontId="10" fillId="2" borderId="0"/>
-    <xf numFmtId="191" fontId="10" fillId="2" borderId="0"/>
     <xf numFmtId="193" fontId="10" fillId="2" borderId="0"/>
-    <xf numFmtId="194" fontId="10" fillId="2" borderId="0" applyAlignment="1">
+    <xf numFmtId="194" fontId="10" fillId="2" borderId="0"/>
+    <xf numFmtId="193" fontId="10" fillId="2" borderId="0"/>
+    <xf numFmtId="195" fontId="10" fillId="2" borderId="0"/>
+    <xf numFmtId="196" fontId="10" fillId="2" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="195" fontId="11" fillId="0" borderId="0"/>
+    <xf numFmtId="197" fontId="11" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="196" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="198" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="0"/>
@@ -1482,7 +1491,7 @@
     <xf numFmtId="0" fontId="15" fillId="20" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="0"/>
-    <xf numFmtId="197" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="199" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="38" fontId="17" fillId="0" borderId="0" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
@@ -1491,10 +1500,10 @@
       <alignment horizontal="centerContinuous"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="21" borderId="5"/>
-    <xf numFmtId="197" fontId="17" fillId="0" borderId="0" applyProtection="1">
+    <xf numFmtId="199" fontId="17" fillId="0" borderId="0" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="197" fontId="17" fillId="0" borderId="6"/>
+    <xf numFmtId="199" fontId="17" fillId="0" borderId="6"/>
     <xf numFmtId="0" fontId="21" fillId="22" borderId="7"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1512,35 +1521,35 @@
     <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="198" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="200" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
     <xf numFmtId="7" fontId="26" fillId="0" borderId="0"/>
     <xf numFmtId="5" fontId="23" fillId="0" borderId="0"/>
-    <xf numFmtId="199" fontId="13" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="201" fontId="13" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="200" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="202" fontId="10" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="201" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="203" fontId="10" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="200" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="202" fontId="10" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="15" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="202" fontId="25" fillId="24" borderId="0"/>
-    <xf numFmtId="203" fontId="27" fillId="0" borderId="8"/>
+    <xf numFmtId="204" fontId="25" fillId="24" borderId="0"/>
+    <xf numFmtId="205" fontId="27" fillId="0" borderId="8"/>
     <xf numFmtId="14" fontId="28" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="204" fontId="28" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="206" fontId="28" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="205" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="207" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="8" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="6" fontId="17" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1548,48 +1557,48 @@
     <xf numFmtId="6" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="39" fontId="10" fillId="25" borderId="0"/>
     <xf numFmtId="7" fontId="10" fillId="25" borderId="0"/>
-    <xf numFmtId="206" fontId="10" fillId="25" borderId="0"/>
-    <xf numFmtId="207" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="208" fontId="10" fillId="25" borderId="0"/>
-    <xf numFmtId="209" fontId="10" fillId="25" borderId="0"/>
-    <xf numFmtId="210" fontId="18" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="211" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="209" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="210" fontId="10" fillId="25" borderId="0"/>
+    <xf numFmtId="211" fontId="10" fillId="25" borderId="0"/>
     <xf numFmtId="212" fontId="18" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="213" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
-    <xf numFmtId="195" fontId="10" fillId="0" borderId="10"/>
-    <xf numFmtId="214" fontId="10" fillId="2" borderId="9" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="215" fontId="10" fillId="2" borderId="9" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="214" fontId="10" fillId="2" borderId="9" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="216" fontId="17" fillId="0" borderId="0" applyProtection="1">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="0"/>
-    <xf numFmtId="217" fontId="31" fillId="0" borderId="0"/>
-    <xf numFmtId="195" fontId="32" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="213" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="214" fontId="18" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="216" fontId="13" fillId="26" borderId="11"/>
+    <xf numFmtId="215" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
+    <xf numFmtId="197" fontId="10" fillId="0" borderId="10"/>
+    <xf numFmtId="216" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="217" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="216" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="218" fontId="17" fillId="0" borderId="0" applyProtection="1">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="0"/>
+    <xf numFmtId="219" fontId="31" fillId="0" borderId="0"/>
+    <xf numFmtId="197" fontId="32" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="218" fontId="13" fillId="26" borderId="11"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="12"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="13"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="14"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0"/>
-    <xf numFmtId="216" fontId="36" fillId="0" borderId="0"/>
+    <xf numFmtId="218" fontId="36" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0"/>
-    <xf numFmtId="197" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="199" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="38" fontId="17" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
@@ -1603,7 +1612,7 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="17" fontId="39" fillId="27" borderId="0"/>
-    <xf numFmtId="218" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="220" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -1614,26 +1623,26 @@
     <xf numFmtId="173" fontId="17" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="219" fontId="10" fillId="0" borderId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="220" fontId="10" fillId="25" borderId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="221" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="219" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="222" fontId="10" fillId="25" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="195" fontId="42" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="223" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="195" fontId="42" fillId="0" borderId="0"/>
-    <xf numFmtId="222" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="221" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="223" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="197" fontId="42" fillId="0" borderId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="197" fontId="42" fillId="0" borderId="0"/>
+    <xf numFmtId="224" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="225" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="1" hidden="1"/>
@@ -1642,62 +1651,62 @@
     <xf numFmtId="37" fontId="26" fillId="0" borderId="0"/>
     <xf numFmtId="175" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="39" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="224" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="226" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
-    <xf numFmtId="225" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="227" fontId="25" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="29" borderId="17"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
-    <xf numFmtId="226" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="228" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="44" fillId="21" borderId="18"/>
-    <xf numFmtId="227" fontId="17" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="229" fontId="17" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
-    <xf numFmtId="228" fontId="10" fillId="25" borderId="0"/>
+    <xf numFmtId="230" fontId="10" fillId="25" borderId="0"/>
     <xf numFmtId="9" fontId="17" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="229" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="231" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="191" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="230" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="231" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="193" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="232" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="233" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="217" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="219" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="8" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="197" fontId="17" fillId="0" borderId="0" applyProtection="1">
+    <xf numFmtId="199" fontId="17" fillId="0" borderId="0" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="216" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="218" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="38" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="193" fontId="10" fillId="2" borderId="19" applyAlignment="1">
+    <xf numFmtId="195" fontId="10" fillId="2" borderId="19" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="232" fontId="46" fillId="2" borderId="0"/>
-    <xf numFmtId="233" fontId="10" fillId="2" borderId="0"/>
+    <xf numFmtId="234" fontId="46" fillId="2" borderId="0"/>
+    <xf numFmtId="235" fontId="10" fillId="2" borderId="0"/>
     <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="8" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="234" fontId="10" fillId="2" borderId="0" applyAlignment="1">
+    <xf numFmtId="236" fontId="10" fillId="2" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="235" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="237" fontId="10" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="236" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="238" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="216" fontId="28" fillId="0" borderId="0"/>
+    <xf numFmtId="218" fontId="28" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1705,10 +1714,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="1" hidden="1"/>
     </xf>
-    <xf numFmtId="197" fontId="17" fillId="0" borderId="0" applyProtection="1">
+    <xf numFmtId="199" fontId="17" fillId="0" borderId="0" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="237" fontId="28" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="239" fontId="28" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="38" fontId="12" fillId="0" borderId="0"/>
@@ -1726,40 +1735,40 @@
     <xf numFmtId="0" fontId="54" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="238" fontId="55" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="240" fontId="55" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="239" fontId="55" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="241" fontId="55" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="25" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="209" fontId="56" fillId="0" borderId="0"/>
-    <xf numFmtId="240" fontId="57" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="211" fontId="56" fillId="0" borderId="0"/>
+    <xf numFmtId="242" fontId="57" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="240" fontId="57" fillId="0" borderId="0"/>
-    <xf numFmtId="240" fontId="58" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="242" fontId="57" fillId="0" borderId="0"/>
+    <xf numFmtId="242" fontId="58" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="240" fontId="58" fillId="0" borderId="0" applyProtection="1">
+    <xf numFmtId="242" fontId="58" fillId="0" borderId="0" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="216" fontId="17" fillId="0" borderId="0" applyProtection="1">
+    <xf numFmtId="218" fontId="17" fillId="0" borderId="0" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="216" fontId="56" fillId="0" borderId="0"/>
+    <xf numFmtId="218" fontId="56" fillId="0" borderId="0"/>
     <xf numFmtId="49" fontId="59" fillId="0" borderId="0"/>
-    <xf numFmtId="241" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="242" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="243" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="244" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="60" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="61" fillId="1" borderId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="216" fontId="62" fillId="0" borderId="0"/>
+    <xf numFmtId="218" fontId="62" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="38" fontId="63" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1768,10 +1777,10 @@
     <xf numFmtId="0" fontId="65" fillId="0" borderId="21"/>
     <xf numFmtId="0" fontId="66" fillId="0" borderId="0"/>
     <xf numFmtId="1" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="243" fontId="26" fillId="0" borderId="0"/>
-    <xf numFmtId="237" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="245" fontId="26" fillId="0" borderId="0"/>
+    <xf numFmtId="239" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="556">
+  <cellXfs count="563">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2503,14 +2512,14 @@
     <xf numFmtId="0" fontId="99" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="100" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="101" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="244" fontId="101" fillId="34" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="190" fontId="101" fillId="34" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="101" fillId="34" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="101" fillId="34" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="102" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="101" fillId="36" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="244" fontId="101" fillId="36" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="245" fontId="101" fillId="34" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="245" fontId="101" fillId="36" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="190" fontId="101" fillId="36" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="191" fontId="101" fillId="34" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="191" fontId="101" fillId="36" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="100" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="101" fillId="36" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="103" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2749,6 +2758,17 @@
     <xf numFmtId="183" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="190" fontId="101" fillId="34" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="102" fillId="35" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="105" fillId="37" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="190" fontId="101" fillId="36" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="191" fontId="101" fillId="34" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="191" fontId="101" fillId="36" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="106" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="187">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3097,6 +3117,127 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>ZoomInfo LBOMODEL1 — Base vs AI-SDR Strategy</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Strategy_Summary'!C49</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Strategy_Summary'!$B$50:$B$55</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Strategy_Summary'!$C$50:$C$55</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Strategy_Summary'!D49</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Strategy_Summary'!$B$50:$B$55</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Strategy_Summary'!$D$50:$D$55</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Value</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -4165,6 +4306,33 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>56</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>1</col>
@@ -4797,14 +4965,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E45"/>
+  <dimension ref="B2:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="48" customWidth="1" style="244" min="2" max="2"/>
     <col width="16" customWidth="1" style="244" min="3" max="3"/>
     <col width="16" customWidth="1" style="244" min="4" max="4"/>
     <col width="14" customWidth="1" style="244" min="5" max="5"/>
-    <col width="40" customWidth="1" style="244" min="6" max="6"/>
+    <col width="78" customWidth="1" style="244" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -4855,7 +5023,7 @@
           <t>Revenue (FY2024)</t>
         </is>
       </c>
-      <c r="C10" s="409" t="n">
+      <c r="C10" s="556" t="n">
         <v>1214.3</v>
       </c>
       <c r="D10" s="408" t="inlineStr">
@@ -4887,7 +5055,7 @@
           <t>GAAP Operating Income</t>
         </is>
       </c>
-      <c r="C12" s="409" t="n">
+      <c r="C12" s="556" t="n">
         <v>97.40000000000001</v>
       </c>
       <c r="D12" s="408" t="inlineStr">
@@ -4902,7 +5070,7 @@
           <t>D&amp;A</t>
         </is>
       </c>
-      <c r="C13" s="409" t="n">
+      <c r="C13" s="556" t="n">
         <v>85.7</v>
       </c>
       <c r="D13" s="408" t="inlineStr">
@@ -4917,7 +5085,7 @@
           <t>Baseline EBITDA (OpInc+D&amp;A)</t>
         </is>
       </c>
-      <c r="C14" s="409" t="n">
+      <c r="C14" s="556" t="n">
         <v>183.1</v>
       </c>
       <c r="D14" s="408" t="inlineStr">
@@ -4947,7 +5115,7 @@
           <t>S&amp;M baseline (35% of rev)</t>
         </is>
       </c>
-      <c r="C16" s="409" t="n">
+      <c r="C16" s="556" t="n">
         <v>425</v>
       </c>
       <c r="D16" s="408" t="inlineStr">
@@ -5013,7 +5181,7 @@
           <t>Sponsor equity check</t>
         </is>
       </c>
-      <c r="C20" s="409" t="n">
+      <c r="C20" s="556" t="n">
         <v>1871.3</v>
       </c>
       <c r="D20" s="408" t="inlineStr">
@@ -5028,7 +5196,7 @@
           <t>New debt (5.0x EBITDA)</t>
         </is>
       </c>
-      <c r="C21" s="409" t="n">
+      <c r="C21" s="556" t="n">
         <v>915.5</v>
       </c>
       <c r="D21" s="408" t="inlineStr">
@@ -5110,8 +5278,13 @@
           <t>Delta</t>
         </is>
       </c>
-    </row>
-    <row r="31">
+      <c r="F30" s="557" t="inlineStr">
+        <is>
+          <t>COMMENTARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="48" customHeight="1" s="244">
       <c r="B31" s="408" t="inlineStr">
         <is>
           <t>Y2 EBITDA margin</t>
@@ -5126,104 +5299,139 @@
       <c r="E31" s="411" t="n">
         <v>0.05519116328280424</v>
       </c>
-    </row>
-    <row r="32">
+      <c r="F31" s="558" t="inlineStr">
+        <is>
+          <t>Year 2 operating profitability; the AI strategy drove this from 15.2% to 20.7%, expanding the margin by 5.5%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="48" customHeight="1" s="244">
       <c r="B32" s="408" t="inlineStr">
         <is>
           <t>Y2 margin vs baseline (bps)</t>
         </is>
       </c>
-      <c r="C32" s="409" t="n">
+      <c r="C32" s="556" t="n">
         <v>14.17277443794801</v>
       </c>
-      <c r="D32" s="414" t="n">
+      <c r="D32" s="559" t="n">
         <v>566.0844072659904</v>
       </c>
-      <c r="E32" s="409" t="n">
+      <c r="E32" s="556" t="n">
         <v>551.9116328280425</v>
       </c>
-    </row>
-    <row r="33">
+      <c r="F32" s="558" t="inlineStr">
+        <is>
+          <t>The difference from baseline margin; AI implementation increased this metric by 551.9 basis points to reach 566.1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="48" customHeight="1" s="244">
       <c r="B33" s="408" t="inlineStr">
         <is>
           <t>Y5 EBITDA ($m)</t>
         </is>
       </c>
-      <c r="C33" s="409" t="n">
+      <c r="C33" s="556" t="n">
         <v>218.4</v>
       </c>
-      <c r="D33" s="414" t="n">
+      <c r="D33" s="559" t="n">
         <v>314.7</v>
       </c>
-      <c r="E33" s="409" t="n">
+      <c r="E33" s="556" t="n">
         <v>96.3</v>
       </c>
-    </row>
-    <row r="34">
+      <c r="F33" s="558" t="inlineStr">
+        <is>
+          <t>Year 5 operating cash flow; AI-driven cost savings boosted this figure by $96.3 million to $314.7 million.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="48" customHeight="1" s="244">
       <c r="B34" s="408" t="inlineStr">
         <is>
           <t>Exit EV @ 13x ($m)</t>
         </is>
       </c>
-      <c r="C34" s="409" t="n">
+      <c r="C34" s="556" t="n">
         <v>2839.7</v>
       </c>
-      <c r="D34" s="414" t="n">
+      <c r="D34" s="559" t="n">
         <v>4091.4</v>
       </c>
-      <c r="E34" s="409" t="n">
+      <c r="E34" s="556" t="n">
         <v>1251.7</v>
       </c>
-    </row>
-    <row r="35">
+      <c r="F34" s="558" t="inlineStr">
+        <is>
+          <t>Projected exit Enterprise Value; higher EBITDA from AI increased this valuation by $1,251.7 million to $4,091.4 million.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="48" customHeight="1" s="244">
       <c r="B35" s="408" t="inlineStr">
         <is>
           <t>Exit net debt ($m)</t>
         </is>
       </c>
-      <c r="C35" s="409" t="n">
+      <c r="C35" s="556" t="n">
         <v>357.1</v>
       </c>
-      <c r="D35" s="414" t="n">
+      <c r="D35" s="559" t="n">
         <v>4.5</v>
       </c>
-      <c r="E35" s="409" t="n">
+      <c r="E35" s="556" t="n">
         <v>-352.6</v>
       </c>
-    </row>
-    <row r="36">
+      <c r="F35" s="558" t="inlineStr">
+        <is>
+          <t>Remaining debt balance at exit; higher cash flow from the AI strategy paid down an extra $352.6 million.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="48" customHeight="1" s="244">
       <c r="B36" s="408" t="inlineStr">
         <is>
           <t>Exit equity value ($m)</t>
         </is>
       </c>
-      <c r="C36" s="409" t="n">
+      <c r="C36" s="556" t="n">
         <v>2482.6</v>
       </c>
-      <c r="D36" s="414" t="n">
+      <c r="D36" s="559" t="n">
         <v>4086.9</v>
       </c>
-      <c r="E36" s="409" t="n">
+      <c r="E36" s="556" t="n">
         <v>1604.3</v>
       </c>
-    </row>
-    <row r="37">
+      <c r="F36" s="558" t="inlineStr">
+        <is>
+          <t>Total payout to equity holders; the AI strategy increased this final payout by $1,604.3 million to $4,086.9 million.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1" s="244">
       <c r="B37" s="408" t="inlineStr">
         <is>
           <t>MOIC</t>
         </is>
       </c>
-      <c r="C37" s="415" t="n">
+      <c r="C37" s="560" t="n">
         <v>1.326661957981033</v>
       </c>
-      <c r="D37" s="416" t="n">
+      <c r="D37" s="561" t="n">
         <v>2.183979483523617</v>
       </c>
-      <c r="E37" s="415" t="n">
+      <c r="E37" s="560" t="n">
         <v>0.8573175255425849</v>
       </c>
-    </row>
-    <row r="38">
+      <c r="F37" s="558" t="inlineStr">
+        <is>
+          <t>Multiple on Invested Capital; the AI strategy significantly improved the total gross cash return from 1.33x to 2.18x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="48" customHeight="1" s="244">
       <c r="B38" s="408" t="inlineStr">
         <is>
           <t>IRR</t>
@@ -5238,6 +5446,18 @@
       <c r="E38" s="411" t="n">
         <v>0.1109330103741204</v>
       </c>
+      <c r="F38" s="558" t="inlineStr">
+        <is>
+          <t>Annualized compound return rate over a 5-year period; replacing human SDRs with AI boosted this return by 11.1 percentage points to 16.9%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="562" t="inlineStr">
+        <is>
+          <t>The IRR is calculated over a 5-year period.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="B40" s="417" t="inlineStr">
@@ -5263,7 +5483,7 @@
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
-          <t>See AI_Operating, Base_Operating, Debt_Sweep_AI, LBO (WSP shell inputs), 00_Assumptions_List</t>
+          <t>See AI_Operating, Base_Operating, Debt_Sweep_AI, LBO, 00_Assumptions_List</t>
         </is>
       </c>
     </row>
@@ -5272,13 +5492,131 @@
         <is>
           <t>10-K: https://www.sec.gov/Archives/edgar/data/1794515/000179451525000045/zi-20241231.htm</t>
         </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>PDF version of this Strategy Summary + Commentary:</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="419" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/vengeanceaiUSC/Rainmaker/cursor/vengeanceaiusclbomodel1-44dc/LBO/output/LBOMODEL1_STRATEGY_SUMMARY.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="407" t="inlineStr">
+        <is>
+          <t>CHART DATA (Base vs AI-SDR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="412" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="C49" s="412" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D49" s="412" t="inlineStr">
+        <is>
+          <t>AI-SDR</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Y2 EBITDA margin %</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="D50" t="n">
+        <v>20.7</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Y5 EBITDA $m</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>218.4</v>
+      </c>
+      <c r="D51" t="n">
+        <v>314.7</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Exit EV $m</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>2839.7</v>
+      </c>
+      <c r="D52" t="n">
+        <v>4091.4</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Exit equity $m</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>2482.6</v>
+      </c>
+      <c r="D53" t="n">
+        <v>4086.9</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>MOIC (x)</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="D54" t="n">
+        <v>2.18</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>IRR %</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="D55" t="n">
+        <v>16.9</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -11319,19 +11657,19 @@
       <c r="B5" s="421" t="n">
         <v>2025</v>
       </c>
-      <c r="C5" s="409" t="n">
+      <c r="C5" s="556" t="n">
         <v>137.5282912000001</v>
       </c>
-      <c r="D5" s="409" t="n">
+      <c r="D5" s="556" t="n">
         <v>137.5282912000001</v>
       </c>
-      <c r="E5" s="414" t="n">
+      <c r="E5" s="559" t="n">
         <v>777.9717088</v>
       </c>
-      <c r="F5" s="409" t="n">
+      <c r="F5" s="556" t="n">
         <v>826.5607773</v>
       </c>
-      <c r="G5" s="414" t="n">
+      <c r="G5" s="559" t="n">
         <v>48.58906850000005</v>
       </c>
     </row>
@@ -11339,19 +11677,19 @@
       <c r="B6" s="421" t="n">
         <v>2026</v>
       </c>
-      <c r="C6" s="409" t="n">
+      <c r="C6" s="556" t="n">
         <v>159.2865991016001</v>
       </c>
-      <c r="D6" s="409" t="n">
+      <c r="D6" s="556" t="n">
         <v>159.2865991016001</v>
       </c>
-      <c r="E6" s="414" t="n">
+      <c r="E6" s="559" t="n">
         <v>618.6851096983999</v>
       </c>
-      <c r="F6" s="409" t="n">
+      <c r="F6" s="556" t="n">
         <v>726.867461747025</v>
       </c>
-      <c r="G6" s="414" t="n">
+      <c r="G6" s="559" t="n">
         <v>108.1823520486251</v>
       </c>
     </row>
@@ -11359,19 +11697,19 @@
       <c r="B7" s="421" t="n">
         <v>2027</v>
       </c>
-      <c r="C7" s="409" t="n">
+      <c r="C7" s="556" t="n">
         <v>183.23549201229</v>
       </c>
-      <c r="D7" s="409" t="n">
+      <c r="D7" s="556" t="n">
         <v>183.23549201229</v>
       </c>
-      <c r="E7" s="414" t="n">
+      <c r="E7" s="559" t="n">
         <v>435.4496176861098</v>
       </c>
-      <c r="F7" s="409" t="n">
+      <c r="F7" s="556" t="n">
         <v>615.320635583216</v>
       </c>
-      <c r="G7" s="414" t="n">
+      <c r="G7" s="559" t="n">
         <v>179.8710178971062</v>
       </c>
     </row>
@@ -11379,19 +11717,19 @@
       <c r="B8" s="421" t="n">
         <v>2028</v>
       </c>
-      <c r="C8" s="409" t="n">
+      <c r="C8" s="556" t="n">
         <v>204.2737956388759</v>
       </c>
-      <c r="D8" s="409" t="n">
+      <c r="D8" s="556" t="n">
         <v>204.2737956388759</v>
       </c>
-      <c r="E8" s="414" t="n">
+      <c r="E8" s="559" t="n">
         <v>231.1758220472339</v>
       </c>
-      <c r="F8" s="409" t="n">
+      <c r="F8" s="556" t="n">
         <v>492.2660966390317</v>
       </c>
-      <c r="G8" s="414" t="n">
+      <c r="G8" s="559" t="n">
         <v>261.0902745917978</v>
       </c>
     </row>
@@ -11399,19 +11737,19 @@
       <c r="B9" s="421" t="n">
         <v>2029</v>
       </c>
-      <c r="C9" s="409" t="n">
+      <c r="C9" s="556" t="n">
         <v>226.6632985760825</v>
       </c>
-      <c r="D9" s="409" t="n">
+      <c r="D9" s="556" t="n">
         <v>226.6632985760825</v>
       </c>
-      <c r="E9" s="414" t="n">
+      <c r="E9" s="559" t="n">
         <v>4.512523471151439</v>
       </c>
-      <c r="F9" s="409" t="n">
+      <c r="F9" s="556" t="n">
         <v>357.1352076643299</v>
       </c>
-      <c r="G9" s="414" t="n">
+      <c r="G9" s="559" t="n">
         <v>352.6226841931785</v>
       </c>
     </row>
@@ -11421,7 +11759,7 @@
           <t>New debt at close</t>
         </is>
       </c>
-      <c r="C11" s="409" t="n">
+      <c r="C11" s="556" t="n">
         <v>915.5000000000001</v>
       </c>
     </row>
@@ -11505,22 +11843,22 @@
           <t>Revenue</t>
         </is>
       </c>
-      <c r="C5" s="409" t="n">
+      <c r="C5" s="556" t="n">
         <v>1214.3</v>
       </c>
-      <c r="D5" s="409" t="n">
+      <c r="D5" s="556" t="n">
         <v>1250.729</v>
       </c>
-      <c r="E5" s="409" t="n">
+      <c r="E5" s="556" t="n">
         <v>1300.75816</v>
       </c>
-      <c r="F5" s="409" t="n">
+      <c r="F5" s="556" t="n">
         <v>1352.7884864</v>
       </c>
-      <c r="G5" s="409" t="n">
+      <c r="G5" s="556" t="n">
         <v>1393.372140992</v>
       </c>
-      <c r="H5" s="409" t="n">
+      <c r="H5" s="556" t="n">
         <v>1435.173305221761</v>
       </c>
     </row>
@@ -11530,22 +11868,22 @@
           <t>COGS</t>
         </is>
       </c>
-      <c r="C6" s="409" t="n">
+      <c r="C6" s="556" t="n">
         <v>189.8</v>
       </c>
-      <c r="D6" s="409" t="n">
+      <c r="D6" s="556" t="n">
         <v>195.4939999999999</v>
       </c>
-      <c r="E6" s="409" t="n">
+      <c r="E6" s="556" t="n">
         <v>203.31376</v>
       </c>
-      <c r="F6" s="409" t="n">
+      <c r="F6" s="556" t="n">
         <v>211.4463104</v>
       </c>
-      <c r="G6" s="409" t="n">
+      <c r="G6" s="556" t="n">
         <v>217.789699712</v>
       </c>
-      <c r="H6" s="409" t="n">
+      <c r="H6" s="556" t="n">
         <v>224.32339070336</v>
       </c>
     </row>
@@ -11555,22 +11893,22 @@
           <t>S&amp;M (human)</t>
         </is>
       </c>
-      <c r="C7" s="409" t="n">
+      <c r="C7" s="556" t="n">
         <v>425</v>
       </c>
-      <c r="D7" s="409" t="n">
+      <c r="D7" s="556" t="n">
         <v>437.75515</v>
       </c>
-      <c r="E7" s="409" t="n">
+      <c r="E7" s="556" t="n">
         <v>455.265356</v>
       </c>
-      <c r="F7" s="409" t="n">
+      <c r="F7" s="556" t="n">
         <v>473.47597024</v>
       </c>
-      <c r="G7" s="409" t="n">
+      <c r="G7" s="556" t="n">
         <v>487.6802493472001</v>
       </c>
-      <c r="H7" s="409" t="n">
+      <c r="H7" s="556" t="n">
         <v>502.3106568276161</v>
       </c>
     </row>
@@ -11580,22 +11918,22 @@
           <t>AI agent cost</t>
         </is>
       </c>
-      <c r="C8" s="409" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="409" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="409" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="409" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="409" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="409" t="n">
+      <c r="C8" s="556" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="556" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="556" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="556" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="556" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="556" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11605,22 +11943,22 @@
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="C9" s="409" t="n">
+      <c r="C9" s="556" t="n">
         <v>196.1</v>
       </c>
-      <c r="D9" s="409" t="n">
+      <c r="D9" s="556" t="n">
         <v>201.983</v>
       </c>
-      <c r="E9" s="409" t="n">
+      <c r="E9" s="556" t="n">
         <v>210.06232</v>
       </c>
-      <c r="F9" s="409" t="n">
+      <c r="F9" s="556" t="n">
         <v>218.4648128</v>
       </c>
-      <c r="G9" s="409" t="n">
+      <c r="G9" s="556" t="n">
         <v>225.018757184</v>
       </c>
-      <c r="H9" s="409" t="n">
+      <c r="H9" s="556" t="n">
         <v>231.7693198995201</v>
       </c>
     </row>
@@ -11630,22 +11968,22 @@
           <t>G&amp;A</t>
         </is>
       </c>
-      <c r="C10" s="409" t="n">
+      <c r="C10" s="556" t="n">
         <v>295.3</v>
       </c>
-      <c r="D10" s="409" t="n">
+      <c r="D10" s="556" t="n">
         <v>225.13122</v>
       </c>
-      <c r="E10" s="409" t="n">
+      <c r="E10" s="556" t="n">
         <v>234.1364688</v>
       </c>
-      <c r="F10" s="409" t="n">
+      <c r="F10" s="556" t="n">
         <v>243.501927552</v>
       </c>
-      <c r="G10" s="409" t="n">
+      <c r="G10" s="556" t="n">
         <v>250.8069853785601</v>
       </c>
-      <c r="H10" s="409" t="n">
+      <c r="H10" s="556" t="n">
         <v>258.3311949399169</v>
       </c>
     </row>
@@ -11655,22 +11993,22 @@
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="C11" s="409" t="n">
+      <c r="C11" s="556" t="n">
         <v>183.1</v>
       </c>
-      <c r="D11" s="414" t="n">
+      <c r="D11" s="559" t="n">
         <v>190.3656300000002</v>
       </c>
-      <c r="E11" s="414" t="n">
+      <c r="E11" s="559" t="n">
         <v>197.9802552000001</v>
       </c>
-      <c r="F11" s="414" t="n">
+      <c r="F11" s="559" t="n">
         <v>205.8994654080003</v>
       </c>
-      <c r="G11" s="414" t="n">
+      <c r="G11" s="559" t="n">
         <v>212.0764493702403</v>
       </c>
-      <c r="H11" s="414" t="n">
+      <c r="H11" s="559" t="n">
         <v>218.4387428513474</v>
       </c>
     </row>
@@ -11705,22 +12043,22 @@
           <t>D&amp;A</t>
         </is>
       </c>
-      <c r="C13" s="409" t="n">
+      <c r="C13" s="556" t="n">
         <v>85.7</v>
       </c>
-      <c r="D13" s="409" t="n">
+      <c r="D13" s="556" t="n">
         <v>88.271</v>
       </c>
-      <c r="E13" s="409" t="n">
+      <c r="E13" s="556" t="n">
         <v>91.80184</v>
       </c>
-      <c r="F13" s="409" t="n">
+      <c r="F13" s="556" t="n">
         <v>95.47391360000002</v>
       </c>
-      <c r="G13" s="409" t="n">
+      <c r="G13" s="556" t="n">
         <v>98.33813100800002</v>
       </c>
-      <c r="H13" s="409" t="n">
+      <c r="H13" s="556" t="n">
         <v>101.28827493824</v>
       </c>
     </row>
@@ -11730,22 +12068,22 @@
           <t>EBIT</t>
         </is>
       </c>
-      <c r="C14" s="409" t="n">
+      <c r="C14" s="556" t="n">
         <v>97.40000000000001</v>
       </c>
-      <c r="D14" s="409" t="n">
+      <c r="D14" s="556" t="n">
         <v>102.0946300000002</v>
       </c>
-      <c r="E14" s="409" t="n">
+      <c r="E14" s="556" t="n">
         <v>106.1784152000001</v>
       </c>
-      <c r="F14" s="409" t="n">
+      <c r="F14" s="556" t="n">
         <v>110.4255518080002</v>
       </c>
-      <c r="G14" s="409" t="n">
+      <c r="G14" s="556" t="n">
         <v>113.7383183622403</v>
       </c>
-      <c r="H14" s="409" t="n">
+      <c r="H14" s="556" t="n">
         <v>117.1504679131074</v>
       </c>
     </row>
@@ -11755,19 +12093,19 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="D15" s="409" t="n">
+      <c r="D15" s="556" t="n">
         <v>68.66250000000001</v>
       </c>
-      <c r="E15" s="409" t="n">
+      <c r="E15" s="556" t="n">
         <v>61.9920582975</v>
       </c>
-      <c r="F15" s="409" t="n">
+      <c r="F15" s="556" t="n">
         <v>54.51505963102687</v>
       </c>
-      <c r="G15" s="409" t="n">
+      <c r="G15" s="556" t="n">
         <v>46.1490476687412</v>
       </c>
-      <c r="H15" s="409" t="n">
+      <c r="H15" s="556" t="n">
         <v>36.91995724792738</v>
       </c>
     </row>
@@ -11777,19 +12115,19 @@
           <t>Net income</t>
         </is>
       </c>
-      <c r="D16" s="409" t="n">
+      <c r="D16" s="556" t="n">
         <v>26.41138270000011</v>
       </c>
-      <c r="E16" s="409" t="n">
+      <c r="E16" s="556" t="n">
         <v>34.90722195297506</v>
       </c>
-      <c r="F16" s="409" t="n">
+      <c r="F16" s="556" t="n">
         <v>44.16928881980895</v>
       </c>
-      <c r="G16" s="409" t="n">
+      <c r="G16" s="556" t="n">
         <v>53.39552384786428</v>
       </c>
-      <c r="H16" s="409" t="n">
+      <c r="H16" s="556" t="n">
         <v>63.38210342549219</v>
       </c>
     </row>
@@ -11799,19 +12137,19 @@
           <t>FCF (after interest)</t>
         </is>
       </c>
-      <c r="D17" s="414" t="n">
+      <c r="D17" s="559" t="n">
         <v>88.93922270000012</v>
       </c>
-      <c r="E17" s="414" t="n">
+      <c r="E17" s="559" t="n">
         <v>99.69331555297505</v>
       </c>
-      <c r="F17" s="414" t="n">
+      <c r="F17" s="559" t="n">
         <v>111.546826163809</v>
       </c>
-      <c r="G17" s="414" t="n">
+      <c r="G17" s="559" t="n">
         <v>123.0545389441843</v>
       </c>
-      <c r="H17" s="414" t="n">
+      <c r="H17" s="559" t="n">
         <v>135.1308889747018</v>
       </c>
     </row>
@@ -11821,19 +12159,19 @@
           <t>Debt paydown</t>
         </is>
       </c>
-      <c r="D18" s="409" t="n">
+      <c r="D18" s="556" t="n">
         <v>88.93922270000012</v>
       </c>
-      <c r="E18" s="409" t="n">
+      <c r="E18" s="556" t="n">
         <v>99.69331555297505</v>
       </c>
-      <c r="F18" s="409" t="n">
+      <c r="F18" s="556" t="n">
         <v>111.546826163809</v>
       </c>
-      <c r="G18" s="409" t="n">
+      <c r="G18" s="556" t="n">
         <v>123.0545389441843</v>
       </c>
-      <c r="H18" s="409" t="n">
+      <c r="H18" s="556" t="n">
         <v>135.1308889747018</v>
       </c>
     </row>
@@ -11843,22 +12181,22 @@
           <t>Debt end</t>
         </is>
       </c>
-      <c r="C19" s="409" t="n">
+      <c r="C19" s="556" t="n">
         <v>1329.9</v>
       </c>
-      <c r="D19" s="409" t="n">
+      <c r="D19" s="556" t="n">
         <v>826.5607773</v>
       </c>
-      <c r="E19" s="409" t="n">
+      <c r="E19" s="556" t="n">
         <v>726.867461747025</v>
       </c>
-      <c r="F19" s="409" t="n">
+      <c r="F19" s="556" t="n">
         <v>615.320635583216</v>
       </c>
-      <c r="G19" s="409" t="n">
+      <c r="G19" s="556" t="n">
         <v>492.2660966390317</v>
       </c>
-      <c r="H19" s="409" t="n">
+      <c r="H19" s="556" t="n">
         <v>357.1352076643299</v>
       </c>
     </row>
@@ -11932,22 +12270,22 @@
           <t>Revenue</t>
         </is>
       </c>
-      <c r="C5" s="409" t="n">
+      <c r="C5" s="556" t="n">
         <v>1214.3</v>
       </c>
-      <c r="D5" s="409" t="n">
+      <c r="D5" s="556" t="n">
         <v>1250.729</v>
       </c>
-      <c r="E5" s="409" t="n">
+      <c r="E5" s="556" t="n">
         <v>1300.75816</v>
       </c>
-      <c r="F5" s="409" t="n">
+      <c r="F5" s="556" t="n">
         <v>1352.7884864</v>
       </c>
-      <c r="G5" s="409" t="n">
+      <c r="G5" s="556" t="n">
         <v>1393.372140992</v>
       </c>
-      <c r="H5" s="409" t="n">
+      <c r="H5" s="556" t="n">
         <v>1435.173305221761</v>
       </c>
     </row>
@@ -11957,22 +12295,22 @@
           <t>COGS</t>
         </is>
       </c>
-      <c r="C6" s="409" t="n">
+      <c r="C6" s="556" t="n">
         <v>189.8</v>
       </c>
-      <c r="D6" s="409" t="n">
+      <c r="D6" s="556" t="n">
         <v>195.4939999999999</v>
       </c>
-      <c r="E6" s="409" t="n">
+      <c r="E6" s="556" t="n">
         <v>203.31376</v>
       </c>
-      <c r="F6" s="409" t="n">
+      <c r="F6" s="556" t="n">
         <v>211.4463104</v>
       </c>
-      <c r="G6" s="409" t="n">
+      <c r="G6" s="556" t="n">
         <v>217.789699712</v>
       </c>
-      <c r="H6" s="409" t="n">
+      <c r="H6" s="556" t="n">
         <v>224.32339070336</v>
       </c>
     </row>
@@ -11982,22 +12320,22 @@
           <t>S&amp;M (human)</t>
         </is>
       </c>
-      <c r="C7" s="409" t="n">
+      <c r="C7" s="556" t="n">
         <v>425</v>
       </c>
-      <c r="D7" s="409" t="n">
+      <c r="D7" s="556" t="n">
         <v>361.25</v>
       </c>
-      <c r="E7" s="409" t="n">
+      <c r="E7" s="556" t="n">
         <v>368.475</v>
       </c>
-      <c r="F7" s="409" t="n">
+      <c r="F7" s="556" t="n">
         <v>375.8445</v>
       </c>
-      <c r="G7" s="409" t="n">
+      <c r="G7" s="556" t="n">
         <v>383.36139</v>
       </c>
-      <c r="H7" s="409" t="n">
+      <c r="H7" s="556" t="n">
         <v>391.0286178000001</v>
       </c>
     </row>
@@ -12007,22 +12345,22 @@
           <t>AI agent cost</t>
         </is>
       </c>
-      <c r="C8" s="409" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="409" t="n">
+      <c r="C8" s="556" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="556" t="n">
         <v>15</v>
       </c>
-      <c r="E8" s="409" t="n">
+      <c r="E8" s="556" t="n">
         <v>15</v>
       </c>
-      <c r="F8" s="409" t="n">
+      <c r="F8" s="556" t="n">
         <v>15</v>
       </c>
-      <c r="G8" s="409" t="n">
+      <c r="G8" s="556" t="n">
         <v>15</v>
       </c>
-      <c r="H8" s="409" t="n">
+      <c r="H8" s="556" t="n">
         <v>15</v>
       </c>
     </row>
@@ -12032,22 +12370,22 @@
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="C9" s="409" t="n">
+      <c r="C9" s="556" t="n">
         <v>196.1</v>
       </c>
-      <c r="D9" s="409" t="n">
+      <c r="D9" s="556" t="n">
         <v>201.983</v>
       </c>
-      <c r="E9" s="409" t="n">
+      <c r="E9" s="556" t="n">
         <v>210.06232</v>
       </c>
-      <c r="F9" s="409" t="n">
+      <c r="F9" s="556" t="n">
         <v>218.4648128</v>
       </c>
-      <c r="G9" s="409" t="n">
+      <c r="G9" s="556" t="n">
         <v>225.018757184</v>
       </c>
-      <c r="H9" s="409" t="n">
+      <c r="H9" s="556" t="n">
         <v>231.7693198995201</v>
       </c>
     </row>
@@ -12057,22 +12395,22 @@
           <t>G&amp;A</t>
         </is>
       </c>
-      <c r="C10" s="409" t="n">
+      <c r="C10" s="556" t="n">
         <v>295.3</v>
       </c>
-      <c r="D10" s="409" t="n">
+      <c r="D10" s="556" t="n">
         <v>225.13122</v>
       </c>
-      <c r="E10" s="409" t="n">
+      <c r="E10" s="556" t="n">
         <v>234.1364688</v>
       </c>
-      <c r="F10" s="409" t="n">
+      <c r="F10" s="556" t="n">
         <v>243.501927552</v>
       </c>
-      <c r="G10" s="409" t="n">
+      <c r="G10" s="556" t="n">
         <v>250.8069853785601</v>
       </c>
-      <c r="H10" s="409" t="n">
+      <c r="H10" s="556" t="n">
         <v>258.3311949399169</v>
       </c>
     </row>
@@ -12082,22 +12420,22 @@
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="C11" s="409" t="n">
+      <c r="C11" s="556" t="n">
         <v>183.1</v>
       </c>
-      <c r="D11" s="414" t="n">
+      <c r="D11" s="559" t="n">
         <v>251.8707800000001</v>
       </c>
-      <c r="E11" s="414" t="n">
+      <c r="E11" s="559" t="n">
         <v>269.7706112000001</v>
       </c>
-      <c r="F11" s="414" t="n">
+      <c r="F11" s="559" t="n">
         <v>288.5309356480003</v>
       </c>
-      <c r="G11" s="414" t="n">
+      <c r="G11" s="559" t="n">
         <v>301.3953087174403</v>
       </c>
-      <c r="H11" s="414" t="n">
+      <c r="H11" s="559" t="n">
         <v>314.7207818789635</v>
       </c>
     </row>
@@ -12132,22 +12470,22 @@
           <t>D&amp;A</t>
         </is>
       </c>
-      <c r="C13" s="409" t="n">
+      <c r="C13" s="556" t="n">
         <v>85.7</v>
       </c>
-      <c r="D13" s="409" t="n">
+      <c r="D13" s="556" t="n">
         <v>88.271</v>
       </c>
-      <c r="E13" s="409" t="n">
+      <c r="E13" s="556" t="n">
         <v>91.80184</v>
       </c>
-      <c r="F13" s="409" t="n">
+      <c r="F13" s="556" t="n">
         <v>95.47391360000002</v>
       </c>
-      <c r="G13" s="409" t="n">
+      <c r="G13" s="556" t="n">
         <v>98.33813100800002</v>
       </c>
-      <c r="H13" s="409" t="n">
+      <c r="H13" s="556" t="n">
         <v>101.28827493824</v>
       </c>
     </row>
@@ -12157,22 +12495,22 @@
           <t>EBIT</t>
         </is>
       </c>
-      <c r="C14" s="409" t="n">
+      <c r="C14" s="556" t="n">
         <v>97.40000000000001</v>
       </c>
-      <c r="D14" s="409" t="n">
+      <c r="D14" s="556" t="n">
         <v>163.5997800000001</v>
       </c>
-      <c r="E14" s="409" t="n">
+      <c r="E14" s="556" t="n">
         <v>177.9687712000001</v>
       </c>
-      <c r="F14" s="409" t="n">
+      <c r="F14" s="556" t="n">
         <v>193.0570220480002</v>
       </c>
-      <c r="G14" s="409" t="n">
+      <c r="G14" s="556" t="n">
         <v>203.0571777094403</v>
       </c>
-      <c r="H14" s="409" t="n">
+      <c r="H14" s="556" t="n">
         <v>213.4325069407234</v>
       </c>
     </row>
@@ -12182,19 +12520,19 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="D15" s="409" t="n">
+      <c r="D15" s="556" t="n">
         <v>68.66250000000001</v>
       </c>
-      <c r="E15" s="409" t="n">
+      <c r="E15" s="556" t="n">
         <v>58.34787815999999</v>
       </c>
-      <c r="F15" s="409" t="n">
+      <c r="F15" s="556" t="n">
         <v>46.40138322737999</v>
       </c>
-      <c r="G15" s="409" t="n">
+      <c r="G15" s="556" t="n">
         <v>32.65872132645823</v>
       </c>
-      <c r="H15" s="409" t="n">
+      <c r="H15" s="556" t="n">
         <v>17.33818665354254</v>
       </c>
     </row>
@@ -12204,19 +12542,19 @@
           <t>Net income</t>
         </is>
       </c>
-      <c r="D16" s="409" t="n">
+      <c r="D16" s="556" t="n">
         <v>75.0004512000001</v>
       </c>
-      <c r="E16" s="409" t="n">
+      <c r="E16" s="556" t="n">
         <v>94.50050550160006</v>
       </c>
-      <c r="F16" s="409" t="n">
+      <c r="F16" s="556" t="n">
         <v>115.85795466829</v>
       </c>
-      <c r="G16" s="409" t="n">
+      <c r="G16" s="556" t="n">
         <v>134.6147805425558</v>
       </c>
-      <c r="H16" s="409" t="n">
+      <c r="H16" s="556" t="n">
         <v>154.9145130268729</v>
       </c>
     </row>
@@ -12226,19 +12564,19 @@
           <t>FCF (after interest)</t>
         </is>
       </c>
-      <c r="D17" s="414" t="n">
+      <c r="D17" s="559" t="n">
         <v>137.5282912000001</v>
       </c>
-      <c r="E17" s="414" t="n">
+      <c r="E17" s="559" t="n">
         <v>159.2865991016001</v>
       </c>
-      <c r="F17" s="414" t="n">
+      <c r="F17" s="559" t="n">
         <v>183.23549201229</v>
       </c>
-      <c r="G17" s="414" t="n">
+      <c r="G17" s="559" t="n">
         <v>204.2737956388759</v>
       </c>
-      <c r="H17" s="414" t="n">
+      <c r="H17" s="559" t="n">
         <v>226.6632985760825</v>
       </c>
     </row>
@@ -12248,19 +12586,19 @@
           <t>Debt paydown</t>
         </is>
       </c>
-      <c r="D18" s="409" t="n">
+      <c r="D18" s="556" t="n">
         <v>137.5282912000001</v>
       </c>
-      <c r="E18" s="409" t="n">
+      <c r="E18" s="556" t="n">
         <v>159.2865991016001</v>
       </c>
-      <c r="F18" s="409" t="n">
+      <c r="F18" s="556" t="n">
         <v>183.23549201229</v>
       </c>
-      <c r="G18" s="409" t="n">
+      <c r="G18" s="556" t="n">
         <v>204.2737956388759</v>
       </c>
-      <c r="H18" s="409" t="n">
+      <c r="H18" s="556" t="n">
         <v>226.6632985760825</v>
       </c>
     </row>
@@ -12270,22 +12608,22 @@
           <t>Debt end</t>
         </is>
       </c>
-      <c r="C19" s="409" t="n">
+      <c r="C19" s="556" t="n">
         <v>1329.9</v>
       </c>
-      <c r="D19" s="409" t="n">
+      <c r="D19" s="556" t="n">
         <v>777.9717088</v>
       </c>
-      <c r="E19" s="409" t="n">
+      <c r="E19" s="556" t="n">
         <v>618.6851096983999</v>
       </c>
-      <c r="F19" s="409" t="n">
+      <c r="F19" s="556" t="n">
         <v>435.4496176861098</v>
       </c>
-      <c r="G19" s="409" t="n">
+      <c r="G19" s="556" t="n">
         <v>231.1758220472339</v>
       </c>
-      <c r="H19" s="409" t="n">
+      <c r="H19" s="556" t="n">
         <v>4.512523471151439</v>
       </c>
     </row>
@@ -13098,7 +13436,6 @@
         <v>134.838525</v>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
@@ -15269,7 +15606,6 @@
         <v>987.5822307314286</v>
       </c>
     </row>
-    <row r="124"/>
     <row r="125">
       <c r="B125" t="inlineStr">
         <is>
@@ -15336,7 +15672,6 @@
         <v>-223</v>
       </c>
     </row>
-    <row r="128"/>
     <row r="129">
       <c r="B129" t="inlineStr">
         <is>
@@ -15878,7 +16213,6 @@
         <v>586.7181807314284</v>
       </c>
     </row>
-    <row r="154"/>
     <row r="155">
       <c r="B155" s="34" t="inlineStr">
         <is>
@@ -16017,7 +16351,6 @@
         </is>
       </c>
     </row>
-    <row r="160"/>
     <row r="161">
       <c r="B161" s="321" t="inlineStr">
         <is>
@@ -19391,7 +19724,6 @@
         <v>0.2849090713511313</v>
       </c>
     </row>
-    <row r="318"/>
     <row r="319">
       <c r="B319" s="317" t="inlineStr">
         <is>
@@ -21880,7 +22212,6 @@
         <v>0.7748616857223557</v>
       </c>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
@@ -22293,7 +22624,6 @@
         <v>36.4886239211832</v>
       </c>
     </row>
-    <row r="82"/>
     <row r="83" ht="17.25" customHeight="1" s="244">
       <c r="C83" s="112" t="inlineStr">
         <is>
@@ -22469,7 +22799,6 @@
       <c r="D93" s="93" t="n"/>
       <c r="E93" s="93" t="n"/>
     </row>
-    <row r="94"/>
     <row r="114">
       <c r="B114" s="108" t="n"/>
       <c r="C114" s="109" t="inlineStr">

</xml_diff>